<commit_message>
feat(productos): Plan de Negocio Bar-Restaurante v2.0 (representante línea A) LIVE — plan financiero como MODELO: hoja 0. Supuestos, tesorería 12 meses y financiación con cuadro francés nuevas, personal = hoja Personal (33,66 %), sin doble conteo de bebida, IS 15 % con BINs, break-even único con cuota y amortización (62,93 cubiertos/día de caja), existencias fuera de la amortización, 766 fórmulas, gates 13/13 (incl. blancos contaminados), checklist 64 ítems con desplegable; docx pendiente de T9
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kK9BRAxpAsfsxudgwH42U
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-bar-restaurante/checklist-apertura-bar-restaurante.xlsx
+++ b/astro-site/public/dl/plan-negocio-bar-restaurante/checklist-apertura-bar-restaurante.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist Apertura" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Checklist Apertura'!$3:$3</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +63,21 @@
       <color rgb="00888888"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000A0908"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +94,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F7F3EC"/>
         <bgColor rgb="00F7F3EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -176,16 +195,64 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C8E6C9"/>
           <bgColor rgb="00C8E6C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -551,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -565,14 +632,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ChefBusiness Consultoria Gastronomica</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Checklist Apertura — Bar-Restaurante / Espana 2026</t>
+          <t>ChefBusiness Consultoría Gastronómica</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Checklist Apertura — Bar-Restaurante / España 2026</t>
         </is>
       </c>
     </row>
@@ -584,7 +651,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Tramite / Tarea</t>
+          <t>Trámite / Tarea</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -608,10 +675,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>FASE 1: CONSTITUCION EMPRESA (Mes 1-2)</t>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>FASE 1: CONSTITUCIÓN DE LA EMPRESA (meses 1-2)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n"/>
@@ -620,7 +687,7 @@
       <c r="E4" s="8" t="n"/>
       <c r="F4" s="9" t="n"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Legal</t>
@@ -628,12 +695,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Elegir forma juridica (SL recomendada, capital min 1 EUR)</t>
+          <t>Elegir forma jurídica (SL recomendada, capital mín. 1 €)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -641,14 +708,14 @@
           <t>Semana 1</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr"/>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Ley Crea y Crece 2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
+          <t>Ley 18/2022 (Crea y Crece): capital mínimo 1 €, con la obligación de destinar el 20 % del beneficio a reserva legal hasta que capital y reserva sumen 3.000 €, y responsabilidad solidaria de los socios por esa diferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Legal</t>
@@ -656,20 +723,20 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Solicitar certificacion negativa de denominacion social</t>
+          <t>Solicitar certificación negativa de denominación social</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>3-5 dias</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
+          <t>3-5 días</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Registro Mercantil Central</t>
@@ -694,10 +761,10 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Depositar capital social</t>
@@ -712,7 +779,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Escritura publica de constitucion ante notario</t>
+          <t>Escritura pública de constitución ante notario</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -722,13 +789,13 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr"/>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>~300-500 EUR</t>
+          <t>~300-500 €</t>
         </is>
       </c>
     </row>
@@ -740,23 +807,23 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Inscripcion en el Registro Mercantil</t>
+          <t>Inscripción en el Registro Mercantil</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>15 dias</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr"/>
+          <t>15 días</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>~150-200 EUR</t>
+          <t>~150-200 €</t>
         </is>
       </c>
     </row>
@@ -773,22 +840,22 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr"/>
       <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Agencia Tributaria</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="135" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Fiscal</t>
@@ -796,23 +863,23 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Alta en el IAE (epigrafe 671.4 restaurantes)</t>
+          <t>Alta en el IAE: epígrafe 671.4 (restaurantes de dos tenedores) o 673.1 (servicios de bar especiales), según el peso de la barra</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Exento si facturacion &lt;1M EUR</t>
+          <t>Doble exención: los dos primeros períodos impositivos de la actividad (art. 82.1.b del TRLRHL) y, después, mientras la cifra de negocio no llegue al millón de euros. La elección del epígrafe la valida tu gestor: condiciona inspecciones y licencia</t>
         </is>
       </c>
     </row>
@@ -824,23 +891,23 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Alta censal y eleccion regimen IVA</t>
+          <t>Alta censal y elección régimen IVA</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr"/>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Regimen general o recargo</t>
+          <t>Régimen general o recargo</t>
         </is>
       </c>
     </row>
@@ -852,23 +919,23 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Inscripcion empresa en Seguridad Social</t>
+          <t>Inscripción empresa en Seguridad Social</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>3 dias</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr"/>
+          <t>3 días</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Codigo cuenta cotizacion</t>
+          <t>Código cuenta cotización</t>
         </is>
       </c>
     </row>
@@ -880,30 +947,30 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Alta autonomos socios trabajadores (si aplica)</t>
+          <t>Alta autónomos socios trabajadores (si aplica)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr"/>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Tarifa plana 80 EUR/mes</t>
+          <t>Tarifa plana 80 €/mes</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>FASE 2: LOCAL Y LICENCIAS (Mes 2-4)</t>
+          <t>FASE 2: LOCAL Y LICENCIAS (meses 2-6)</t>
         </is>
       </c>
       <c r="B15" s="8" t="n"/>
@@ -920,7 +987,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Busqueda y negociacion del local</t>
+          <t>Búsqueda y negociación del local</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -933,14 +1000,14 @@
           <t>2-4 semanas</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr"/>
+      <c r="E16" s="12" t="inlineStr"/>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Verificar uso hosteleria permitido</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+          <t>Verificar uso hostelería permitido</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Local</t>
@@ -958,13 +1025,13 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr"/>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Revisar clausulas: duracion, renta, obras</t>
+          <t>Revisar cláusulas: duración, renta, obras</t>
         </is>
       </c>
     </row>
@@ -976,7 +1043,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Declaracion responsable o licencia actividad</t>
+          <t>Declaración responsable o licencia actividad</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -989,14 +1056,14 @@
           <t>1-3 meses</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr"/>
+      <c r="E18" s="12" t="inlineStr"/>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Segun municipio</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
+          <t>Según municipio</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Licencia</t>
@@ -1004,12 +1071,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Proyecto tecnico de actividad (ingeniero/arquitecto)</t>
+          <t>Proyecto técnico de actividad (ingeniero/arquitecto)</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Tecnico</t>
+          <t>Técnico</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1017,7 +1084,7 @@
           <t>2-4 semanas</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr"/>
+      <c r="E19" s="12" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Incluye APPCC, accesibilidad, incendios</t>
@@ -1045,14 +1112,14 @@
           <t>1-2 meses</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr"/>
+      <c r="E20" s="12" t="inlineStr"/>
       <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Depende de la obra</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Licencia</t>
@@ -1060,12 +1127,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Autorizacion sanitaria de funcionamiento</t>
+          <t>Inscripción en el Registro Sanitario de tu Comunidad Autónoma (declaración responsable de inicio de actividad alimentaria)</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Consejeria</t>
+          <t>Consejería</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1073,10 +1140,10 @@
           <t>2-4 semanas</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr"/>
+      <c r="E21" s="12" t="inlineStr"/>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Registro RGSEAA</t>
+          <t>El Registro General Sanitario estatal NO aplica al minorista que sirve al consumidor final (art. 2.2 del RD 191/2011): el que te toca es el autonómico</t>
         </is>
       </c>
     </row>
@@ -1088,23 +1155,23 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Inscripcion Registro General Sanitario</t>
+          <t>Licencia de terraza (si aplica)</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Comunidad</t>
+          <t>Ayuntamiento</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>2-4 semanas</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr"/>
+          <t>1-3 meses</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr"/>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Obligatorio para servir alimentos</t>
+          <t>Tasa anual + m2</t>
         </is>
       </c>
     </row>
@@ -1116,67 +1183,67 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Licencia de terraza (si aplica)</t>
+          <t>Alta suministros: luz, agua, gas</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Ayuntamiento</t>
+          <t>Socios</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>1-3 meses</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr"/>
+          <t>1-2 semanas</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Tasa anual + m2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Licencia</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Alta suministros: luz, agua, gas</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Socios</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>1-2 semanas</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
           <t>Contratos a nombre de la sociedad</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>FASE 3: OBRA Y EQUIPAMIENTO (Mes 3-5)</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="22" customHeight="1">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>FASE 3: OBRA Y EQUIPAMIENTO (meses 4-7)</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Obra</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Reforma y acondicionamiento del local</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Contratista</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>4-8 semanas</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Según proyecto técnico</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Obra</t>
@@ -1184,51 +1251,51 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Reforma y acondicionamiento del local</t>
+          <t>Instalación cocina: extracción, gas, electricidad</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Contratista</t>
+          <t>Instalador</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>4-8 semanas</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr"/>
+          <t>2-3 semanas</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr"/>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Segun proyecto tecnico</t>
+          <t>Certificados instalación</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Obra</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Instalacion cocina: extraccion, gas, electricidad</t>
+          <t>Compra e instalación equipamiento cocina</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Instalador</t>
+          <t>Socios</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>2-3 semanas</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr"/>
+          <t>2 semanas</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr"/>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Certificados instalacion</t>
+          <t>Ver hoja Inversión Inicial</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1307,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Compra e instalacion equipamiento cocina</t>
+          <t>Compra mobiliario sala y barra</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1253,12 +1320,8 @@
           <t>2 semanas</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Ver hoja Inversion Inicial</t>
-        </is>
-      </c>
+      <c r="E28" s="12" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1268,21 +1331,25 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Compra mobiliario sala y barra</t>
+          <t>Instalación TPV y software hostelería</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Socios</t>
+          <t>Proveedor</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>2 semanas</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="6" t="inlineStr"/>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Formación equipo incluida</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1292,7 +1359,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Instalacion TPV y software hosteleria</t>
+          <t>Instalación cafetera y grifos cerveza</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1302,41 +1369,41 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr"/>
+          <t>1-2 días</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Formacion equipo incluida</t>
+          <t>Servicio técnico oficial</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>APPCC</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Instalacion cafetera y grifos cerveza</t>
+          <t>Implementar sistema APPCC completo</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Proveedor</t>
+          <t>Consultor</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>1-2 dias</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr"/>
+          <t>2 semanas</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Servicio tecnico oficial</t>
+          <t>Plan autocontrol obligatorio</t>
         </is>
       </c>
     </row>
@@ -1348,65 +1415,65 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Implementar sistema APPCC completo</t>
+          <t>Registro de alérgenos en carta</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Consultor</t>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>14 alérgenos obligatorios UE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>FASE 4: PERSONAL (mes 7)</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Publicar ofertas de empleo</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
           <t>2 semanas</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Plan autocontrol obligatorio</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>APPCC</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Registro de alergenos en carta</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>14 alergenos obligatorios UE</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>FASE 4: PERSONAL (Mes 4-5)</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="n"/>
-      <c r="C34" s="8" t="n"/>
-      <c r="D34" s="8" t="n"/>
-      <c r="E34" s="8" t="n"/>
-      <c r="F34" s="9" t="n"/>
+      <c r="E34" s="12" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>InfoJobs, Indeed, boca a boca</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -1416,7 +1483,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Publicar ofertas de empleo</t>
+          <t>Selección y entrevistas</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -1429,10 +1496,10 @@
           <t>2 semanas</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr"/>
+      <c r="E35" s="12" t="inlineStr"/>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>InfoJobs, Indeed, boca a boca</t>
+          <t>Priorizar experiencia hostelería</t>
         </is>
       </c>
     </row>
@@ -1444,23 +1511,23 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Seleccion y entrevistas</t>
+          <t>Contratos de trabajo</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Socios</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>2 semanas</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr"/>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr"/>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Priorizarcexperiencia hosteleria</t>
+          <t>Convenio hostelería de tu provincia</t>
         </is>
       </c>
     </row>
@@ -1472,25 +1539,21 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Contratos de trabajo</t>
+          <t>Alta trabajadores en Seguridad Social</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Gestoría</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr"/>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>Convenio hosteleria de tu provincia</t>
-        </is>
-      </c>
+          <t>Antes inicio</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -1500,23 +1563,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Alta trabajadores en Seguridad Social</t>
+          <t>Formación equipo: carta, servicio, APPCC</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Gestoria</t>
+          <t>Socios</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Antes inicio</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
+          <t>1-2 semanas</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Antes de abrir</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="75" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
           <t>RRHH</t>
@@ -1524,27 +1591,27 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Formacion equipo: carta, servicio, APPCC</t>
+          <t>Formación en higiene alimentaria de todo el equipo</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Socios</t>
+          <t>Titular</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>1-2 semanas</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr"/>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Antes de abrir</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
+          <t>El «carnet de manipulador» está derogado (RD 109/2010): la formación la acredita la EMPRESA y se documenta en el plan APPCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="120" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
           <t>RRHH</t>
@@ -1552,88 +1619,84 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Carnet de manipulador de alimentos (todo el equipo)</t>
+          <t>Plan de prevención de riesgos laborales (asumido por el titular o con servicio ajeno)</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Empleados</t>
+          <t>Titular o servicio ajeno</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr"/>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr"/>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Obligatorio, online ~15 EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>RRHH</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Prevencion riesgos laborales</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Servicio PRL</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr"/>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>Obligatorio contratar servicio externo</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>FASE 5: MARKETING Y LANZAMIENTO (Mes 5-6)</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="n"/>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
-      <c r="E42" s="8" t="n"/>
-      <c r="F42" s="9" t="n"/>
+          <t>Obligatorio es el PLAN de prevención, no contratar un servicio ajeno: con menos de 25 trabajadores y un solo centro el empresario puede asumir la actividad preventiva (art. 30.5 de la Ley 31/1995 y art. 11 del RD 39/1997)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>FASE 5: MARKETING Y LANZAMIENTO (meses 7-8)</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="9" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Diseño logo, identidad visual, carta</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Diseñador</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>2-3 semanas</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Marca</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Diseno logo, identidad visual, carta</t>
+          <t>Crear web básica + dominio</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Disenador</t>
+          <t>Agencia/DIY</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>2-3 semanas</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr"/>
+          <t>1-2 semanas</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr"/>
       <c r="F43" s="6" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
@@ -1644,21 +1707,25 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Crear web basica + dominio</t>
+          <t>Alta Google My Business + fotos profesionales</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Agencia/DIY</t>
+          <t>Socios</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>1-2 semanas</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr"/>
-      <c r="F44" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Crítico para SEO local</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -1668,7 +1735,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Alta Google My Business + fotos profesionales</t>
+          <t>Perfiles RRSS: Instagram, TikTok, Facebook</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -1678,15 +1745,11 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Critico para SEO local</t>
-        </is>
-      </c>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -1696,7 +1759,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Perfiles RRSS: Instagram, TikTok, Facebook</t>
+          <t>Configurar reservas online (TheFork, Google)</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -1706,35 +1769,39 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr"/>
       <c r="F46" s="6" t="inlineStr"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Lanzamiento</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Configurar reservas online (TheFork, Google)</t>
+          <t>Soft opening con familia/amigos (1 semana)</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Socios</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr"/>
-      <c r="F47" s="6" t="inlineStr"/>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Detectar fallos antes de abrir</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -1744,7 +1811,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Soft opening con familia/amigos (1 semana)</t>
+          <t>Inauguración oficial + evento</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -1754,13 +1821,13 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr"/>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr"/>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Detectar fallos antes de abrir</t>
+          <t>Invitar prensa local, influencers</t>
         </is>
       </c>
     </row>
@@ -1772,285 +1839,703 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Inauguracion oficial + evento</t>
+          <t>Activar campaña RRSS + Google Ads local</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Primeras 4 semanas críticas</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>FASE 6: OBLIGACIONES QUE HAY QUE TENER CERRADAS ANTES DE ABRIR (meses 6-8)</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Seguros</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Contratar el seguro de responsabilidad civil y el multirriesgo del local</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>Antes de abrir</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr"/>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Está presupuestado en la hoja de Inversión y hasta ahora no había ninguna tarea que lo ejecutara</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Hojas de reclamaciones oficiales y su cartel anunciador</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr"/>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>El modelo y el texto del cartel los aprueba tu Comunidad Autónoma</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>Laboral</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Registro horario diario de la jornada de todo el equipo</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Gestoría</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>Desde el primer contrato</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr"/>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>Art. 34.9 del Estatuto de los Trabajadores; se conserva cuatro años</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="45" customHeight="1">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Contrato con gestor autorizado de residuos y de aceite vegetal usado</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>2 semanas</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr"/>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>Se comprueba en la inspección; el aceite usado no puede ir al desagüe</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="45" customHeight="1">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>APPCC</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Contrato de desinsectación, desratización y desinfección (DDD)</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="inlineStr"/>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>Empresa inscrita en el ROESB; el certificado forma parte del plan APPCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="45" customHeight="1">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Licencia de derechos de autor por la música ambiental</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>2 semanas</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr"/>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>SGAE y AGEDI-AIE son dos licencias distintas y se pagan las dos</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="45" customHeight="1">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>APPCC</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Plan de prevención de las pérdidas y el desperdicio alimentario</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr"/>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>Ley 1/2025: obliga a tener un plan escrito y a ofrecer la comida sobrante para donación</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="45" customHeight="1">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Obra</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Boletines de la instalación eléctrica y de la instalación de gas</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Instalador</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>Con la obra</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr"/>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>Sin ellos no hay alta de suministros ni licencia de actividad</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="45" customHeight="1">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Laboral</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Comunicación de apertura del centro de trabajo a la autoridad laboral</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>Gestoría</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>Primeros 30 días</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="n"/>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>Se presenta en los treinta días siguientes al inicio de la actividad</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="45" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Cartel de prohibición de venta de alcohol y tabaco a menores</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>1 día</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="n"/>
+      <c r="F60" s="15" t="inlineStr">
+        <is>
+          <t>La redacción exacta y el tamaño los fija tu Comunidad Autónoma</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="75" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>RGPD</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Registro de actividades de tratamiento de datos personales</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>Antes de abrir</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="n"/>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>Art. 30 del RGPD y art. 31 de la LOPDGDD: lo pide la AEPD en la primera inspección. Incluye clientes, personal y proveedores</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="75" customHeight="1">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>RGPD</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Informar al equipo del registro horario y del tratamiento de sus datos</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>Gestoría</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Desde el primer contrato</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>La cláusula informativa se entrega con el contrato; el fichaje es un tratamiento de datos, no sólo una obligación laboral</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="60" customHeight="1">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>RGPD</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>Cartel y contrato de videovigilancia con la empresa de seguridad</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Con la obra</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="n"/>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>Cartel homologado en zona visible, contrato de encargado de tratamiento y plazo máximo de conservación de 30 días</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="60" customHeight="1">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>RGPD</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Cláusula informativa y consentimiento en el sistema de reservas y en la lista de correo</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>Socios</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Antes de abrir</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="n"/>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>Reservas online, WhatsApp y newsletter tratan datos: cada canal necesita su información previa</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="120" customHeight="1">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>Fiscal</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Adaptar el TPV y la facturación al sistema Veri*factu / factura electrónica</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>Gestoría</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>Antes de abrir</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="n"/>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>El RD 1007/2023 y su calendario escalonado obligan a que el software de facturación sea verificable. Consulta la fecha que te aplica antes de comprar el TPV que presupuesta la hoja de Inversión: cambiarlo después cuesta el doble</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
+        <is>
+          <t>FASE 7: PRIMEROS 90 DÍAS (meses 8-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Revisión diaria de ventas y food cost</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Diario</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Ajustar carta según demanda real</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="n"/>
+    </row>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Implementar encuesta satisfacción cliente</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>Evaluar desempeño equipo</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>Financiero</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Revisar P&amp;L vs previsiones</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>Gestoría</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>Financiero</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>Ajustar precios si food cost se desvía</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>Evaluar ROI campaña marketing</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="n"/>
+    </row>
+    <row r="74" ht="15" customHeight="1">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>Pedir reseñas Google a clientes satisfechos</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>1 dia</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr"/>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>Invitar prensa local, influencers</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Lanzamiento</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Activar campana RRSS + Google Ads local</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr"/>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>Primeras 4 semanas criticas</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>FASE 6: PRIMEROS 90 DIAS (Mes 6-8)</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="8" t="n"/>
-      <c r="F51" s="9" t="n"/>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Operacion</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Revision diaria de ventas y food cost</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Gerente</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Diario</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr"/>
-      <c r="F52" s="6" t="inlineStr"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Operacion</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Ajustar carta segun demanda real</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr"/>
-      <c r="F53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Operacion</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Implementar encuesta satisfaccion cliente</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Gerente</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Semanal</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr"/>
-      <c r="F54" s="6" t="inlineStr"/>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Operacion</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Evaluar desempeno equipo</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Gerente</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr"/>
-      <c r="F55" s="6" t="inlineStr"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Financiero</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Revisar P&amp;L vs previsiones</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Gestoria</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr"/>
-      <c r="F56" s="6" t="inlineStr"/>
-    </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Financiero</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>Ajustar precios si food cost se desvía</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>Gerente</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr"/>
-      <c r="F57" s="6" t="inlineStr"/>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Evaluar ROI campanas marketing</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr"/>
-      <c r="F58" s="6" t="inlineStr"/>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Pedir resenas Google a clientes satisfechos</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>Continuo</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr"/>
-      <c r="F59" s="6" t="inlineStr"/>
-    </row>
-    <row r="60"/>
-    <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>ChefBusiness.co — Checklist Apertura Bar-Restaurante / Espana 2026</t>
-        </is>
+      <c r="E74" s="16" t="n"/>
+    </row>
+    <row r="75"/>
+    <row r="76" ht="75" customHeight="1">
+      <c r="A76" s="19" t="inlineStr">
+        <is>
+          <t>ChefBusiness.co — Checklist Apertura Bar-Restaurante / España 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="20" t="inlineStr">
+        <is>
+          <t>Ítems completados:</t>
+        </is>
+      </c>
+      <c r="E77" s="21">
+        <f>COUNTIF(E5:E74,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="G77" s="21">
+        <f>COUNTIF(B5:B74,"?*")-COUNTIF(E5:E74,"N/A")</f>
+        <v>64.0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:F59">
+  <conditionalFormatting sqref="A4:F77">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E4="✓"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E5:E74">
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" stopIfTrue="1" text="✓">
+      <formula>NOT(ISERROR(SEARCH("✓",E5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E16 E17 E18 E19 E20 E21 E22 E23 E24 E26 E27 E28 E29 E30 E31 E32 E33 E35 E36 E37 E38 E39 E40 E41 E43 E44 E45 E46 E47 E48 E49 E50 E52 E53 E54 E55 E56 E57 E58 E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E16 E17 E18 E19 E20 E21 E22 E23 E25 E26 E27 E28 E29 E30 E31 E32 E34 E35 E36 E37 E38 E39 E40 E42 E43 E44 E45 E46 E47 E48 E49 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E67 E68 E69 E70 E71 E72 E73 E74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2065,4 +2550,96 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES DE USO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Este fichero forma parte del producto «plan-negocio-bar-restaurante» de AI Chef Pro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Las celdas VERDES son las editables: cambia esas y el resto del libro se recalcula solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Columna OK: elige ✓ (hecho), — (pendiente) o N/A (no aplica). Las N/A no cuentan en el total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>El contador del pie cuenta sólo las ✓ de toda la lista; las N/A salen del total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Para editar una celda que no esté en verde: Revisar → Desproteger hoja (no tiene contraseña).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Más plantillas y kits del catálogo en aichef.pro/productos-digitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/plan-negocio-bar-restaurante · info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>